<commit_message>
added mlcluster surveyer logic
</commit_message>
<xml_diff>
--- a/data/Direct_Inflation_Estimations_12m.xlsx
+++ b/data/Direct_Inflation_Estimations_12m.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Current\Work\LLMExpectations\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{166AD36A-528D-4DEC-A667-606A9A797FB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BAFF03E-8E9D-4BBF-BEE9-72978E8E611A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{1FAA35AD-736E-47F1-B072-A353E63F22DC}"/>
   </bookViews>
@@ -536,10 +536,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6AA8CF70-0E2E-4BE5-88B6-97F23352F385}">
-  <dimension ref="A1:FE3"/>
+  <dimension ref="A1:FF3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="14" max="14" width="11.26953125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:161" ht="31" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:162" ht="31" x14ac:dyDescent="0.35">
       <c r="A1" s="1"/>
       <c r="B1" s="2">
         <v>40148</v>
@@ -578,451 +581,454 @@
         <v>41244</v>
       </c>
       <c r="N1" s="2">
-        <v>41334</v>
+        <v>41365</v>
       </c>
       <c r="O1" s="2">
-        <v>41426</v>
+        <v>41427</v>
       </c>
       <c r="P1" s="2">
-        <v>41518</v>
+        <v>41526</v>
       </c>
       <c r="Q1" s="2">
-        <v>41609</v>
+        <v>41610</v>
       </c>
       <c r="R1" s="2">
-        <v>41671</v>
+        <v>41673</v>
       </c>
       <c r="S1" s="2">
-        <v>41730</v>
+        <v>41757</v>
       </c>
       <c r="T1" s="2">
-        <v>41760</v>
+        <v>41785</v>
       </c>
       <c r="U1" s="2">
-        <v>41791</v>
+        <v>41813</v>
       </c>
       <c r="V1" s="2">
-        <v>41821</v>
+        <v>41849</v>
       </c>
       <c r="W1" s="2">
-        <v>41852</v>
+        <v>41875</v>
       </c>
       <c r="X1" s="2">
-        <v>41883</v>
+        <v>41904</v>
       </c>
       <c r="Y1" s="2">
-        <v>41913</v>
+        <v>41940</v>
       </c>
       <c r="Z1" s="2">
-        <v>41944</v>
+        <v>41967</v>
       </c>
       <c r="AA1" s="2">
-        <v>41974</v>
+        <v>41988</v>
       </c>
       <c r="AB1" s="2">
-        <v>42005</v>
+        <v>42022</v>
       </c>
       <c r="AC1" s="2">
-        <v>42036</v>
+        <v>42057</v>
       </c>
       <c r="AD1" s="2">
-        <v>42064</v>
+        <v>42085</v>
       </c>
       <c r="AE1" s="2">
-        <v>42095</v>
+        <v>42113</v>
       </c>
       <c r="AF1" s="2">
-        <v>42125</v>
+        <v>42148</v>
       </c>
       <c r="AG1" s="2">
-        <v>42156</v>
+        <v>42176</v>
       </c>
       <c r="AH1" s="2">
-        <v>42186</v>
+        <v>42204</v>
       </c>
       <c r="AI1" s="2">
-        <v>42217</v>
+        <v>42232</v>
       </c>
       <c r="AJ1" s="2">
-        <v>42248</v>
+        <v>42267</v>
       </c>
       <c r="AK1" s="2">
-        <v>42278</v>
+        <v>42295</v>
       </c>
       <c r="AL1" s="2">
-        <v>42309</v>
+        <v>42323</v>
       </c>
       <c r="AM1" s="2">
-        <v>42339</v>
+        <v>42351</v>
       </c>
       <c r="AN1" s="2">
-        <v>42370</v>
+        <v>42388</v>
       </c>
       <c r="AO1" s="2">
-        <v>42401</v>
+        <v>42416</v>
       </c>
       <c r="AP1" s="2">
-        <v>42430</v>
+        <v>42446</v>
       </c>
       <c r="AQ1" s="2">
-        <v>42461</v>
+        <v>42472</v>
       </c>
       <c r="AR1" s="2">
-        <v>42491</v>
+        <v>42506</v>
       </c>
       <c r="AS1" s="2">
-        <v>42522</v>
+        <v>42533</v>
       </c>
       <c r="AT1" s="2">
-        <v>42552</v>
+        <v>42564</v>
       </c>
       <c r="AU1" s="2">
-        <v>42583</v>
+        <v>42598</v>
       </c>
       <c r="AV1" s="2">
-        <v>42614</v>
+        <v>42626</v>
       </c>
       <c r="AW1" s="2">
-        <v>42644</v>
+        <v>42654</v>
       </c>
       <c r="AX1" s="2">
-        <v>42675</v>
+        <v>42682</v>
       </c>
       <c r="AY1" s="2">
-        <v>42705</v>
+        <v>42710</v>
       </c>
       <c r="AZ1" s="2">
-        <v>42736</v>
+        <v>42752</v>
       </c>
       <c r="BA1" s="2">
-        <v>42767</v>
+        <v>42780</v>
       </c>
       <c r="BB1" s="2">
-        <v>42795</v>
+        <v>42804</v>
       </c>
       <c r="BC1" s="2">
-        <v>42826</v>
+        <v>42836</v>
       </c>
       <c r="BD1" s="2">
-        <v>42856</v>
+        <v>42872</v>
       </c>
       <c r="BE1" s="2">
-        <v>42887</v>
+        <v>42899</v>
       </c>
       <c r="BF1" s="2">
-        <v>42917</v>
+        <v>42927</v>
       </c>
       <c r="BG1" s="2">
-        <v>42948</v>
+        <v>42962</v>
       </c>
       <c r="BH1" s="2">
-        <v>42979</v>
+        <v>42990</v>
       </c>
       <c r="BI1" s="2">
-        <v>43009</v>
+        <v>43018</v>
       </c>
       <c r="BJ1" s="2">
-        <v>43040</v>
+        <v>43046</v>
       </c>
       <c r="BK1" s="2">
-        <v>43070</v>
+        <v>43074</v>
       </c>
       <c r="BL1" s="2">
-        <v>43101</v>
+        <v>43123</v>
       </c>
       <c r="BM1" s="2">
-        <v>43132</v>
+        <v>43143</v>
       </c>
       <c r="BN1" s="2">
-        <v>43160</v>
+        <v>43171</v>
       </c>
       <c r="BO1" s="2">
-        <v>43191</v>
+        <v>43199</v>
       </c>
       <c r="BP1" s="2">
-        <v>43221</v>
+        <v>43234</v>
       </c>
       <c r="BQ1" s="2">
-        <v>43252</v>
+        <v>43269</v>
       </c>
       <c r="BR1" s="2">
-        <v>43282</v>
+        <v>43297</v>
       </c>
       <c r="BS1" s="2">
-        <v>43313</v>
+        <v>43325</v>
       </c>
       <c r="BT1" s="2">
-        <v>43344</v>
+        <v>43353</v>
       </c>
       <c r="BU1" s="2">
-        <v>43374</v>
+        <v>43381</v>
       </c>
       <c r="BV1" s="2">
-        <v>43405</v>
+        <v>43416</v>
       </c>
       <c r="BW1" s="2">
-        <v>43435</v>
+        <v>43444</v>
       </c>
       <c r="BX1" s="2">
-        <v>43466</v>
+        <v>43483</v>
       </c>
       <c r="BY1" s="2">
-        <v>43497</v>
+        <v>43510</v>
       </c>
       <c r="BZ1" s="2">
-        <v>43525</v>
+        <v>43535</v>
       </c>
       <c r="CA1" s="2">
-        <v>43556</v>
+        <v>43566</v>
       </c>
       <c r="CB1" s="2">
-        <v>43586</v>
+        <v>43601</v>
       </c>
       <c r="CC1" s="2">
-        <v>43617</v>
+        <v>43626</v>
       </c>
       <c r="CD1" s="2">
-        <v>43647</v>
+        <v>43657</v>
       </c>
       <c r="CE1" s="2">
-        <v>43678</v>
+        <v>43692</v>
       </c>
       <c r="CF1" s="2">
-        <v>43709</v>
+        <v>43720</v>
       </c>
       <c r="CG1" s="2">
-        <v>43739</v>
+        <v>43748</v>
       </c>
       <c r="CH1" s="2">
-        <v>43770</v>
+        <v>43783</v>
       </c>
       <c r="CI1" s="2">
-        <v>43800</v>
+        <v>43808</v>
       </c>
       <c r="CJ1" s="2">
-        <v>43831</v>
+        <v>43846</v>
       </c>
       <c r="CK1" s="2">
-        <v>43862</v>
+        <v>43873</v>
       </c>
       <c r="CL1" s="2">
-        <v>43891</v>
+        <v>43901</v>
       </c>
       <c r="CM1" s="2">
-        <v>44044</v>
+        <v>44055</v>
       </c>
       <c r="CN1" s="2">
-        <v>44075</v>
+        <v>44083</v>
       </c>
       <c r="CO1" s="2">
-        <v>44105</v>
+        <v>44113</v>
       </c>
       <c r="CP1" s="2">
-        <v>44136</v>
+        <v>44147</v>
       </c>
       <c r="CQ1" s="2">
-        <v>44166</v>
+        <v>44175</v>
       </c>
       <c r="CR1" s="2">
-        <v>44197</v>
+        <v>44217</v>
       </c>
       <c r="CS1" s="2">
-        <v>44228</v>
+        <v>44242</v>
       </c>
       <c r="CT1" s="2">
-        <v>44256</v>
+        <v>44266</v>
       </c>
       <c r="CU1" s="2">
-        <v>44287</v>
+        <v>44298</v>
       </c>
       <c r="CV1" s="2">
-        <v>44317</v>
+        <v>44330</v>
       </c>
       <c r="CW1" s="2">
-        <v>44348</v>
+        <v>44358</v>
       </c>
       <c r="CX1" s="2">
-        <v>44378</v>
+        <v>44389</v>
       </c>
       <c r="CY1" s="2">
-        <v>44409</v>
+        <v>44420</v>
       </c>
       <c r="CZ1" s="2">
-        <v>44440</v>
+        <v>44452</v>
       </c>
       <c r="DA1" s="2">
-        <v>44470</v>
+        <v>44480</v>
       </c>
       <c r="DB1" s="2">
-        <v>44501</v>
+        <v>44512</v>
       </c>
       <c r="DC1" s="2">
-        <v>44531</v>
+        <v>44539</v>
       </c>
       <c r="DD1" s="2">
         <v>44581</v>
       </c>
       <c r="DE1" s="2">
-        <v>44607</v>
+        <v>44606</v>
       </c>
       <c r="DF1" s="2">
-        <v>44631</v>
+        <v>44630</v>
       </c>
       <c r="DG1" s="2">
-        <v>44660</v>
+        <v>44659</v>
       </c>
       <c r="DH1" s="2">
-        <v>44694</v>
+        <v>44693</v>
       </c>
       <c r="DI1" s="2">
-        <v>44723</v>
+        <v>44722</v>
       </c>
       <c r="DJ1" s="2">
-        <v>44743</v>
+        <v>44750</v>
       </c>
       <c r="DK1" s="2">
-        <v>44774</v>
+        <v>44784</v>
       </c>
       <c r="DL1" s="2">
-        <v>44805</v>
+        <v>44812</v>
       </c>
       <c r="DM1" s="2">
-        <v>44835</v>
+        <v>44847</v>
       </c>
       <c r="DN1" s="2">
-        <v>44866</v>
+        <v>44876</v>
       </c>
       <c r="DO1" s="2">
-        <v>44896</v>
+        <v>44903</v>
       </c>
       <c r="DP1" s="2">
-        <v>44927</v>
+        <v>44944</v>
       </c>
       <c r="DQ1" s="2">
-        <v>44958</v>
+        <v>44967</v>
       </c>
       <c r="DR1" s="2">
-        <v>44986</v>
+        <v>44995</v>
       </c>
       <c r="DS1" s="2">
-        <v>45017</v>
+        <v>45027</v>
       </c>
       <c r="DT1" s="2">
-        <v>45047</v>
+        <v>45056</v>
       </c>
       <c r="DU1" s="2">
-        <v>45078</v>
+        <v>45090</v>
       </c>
       <c r="DV1" s="2">
-        <v>45108</v>
+        <v>45119</v>
       </c>
       <c r="DW1" s="2">
-        <v>45139</v>
+        <v>45148</v>
       </c>
       <c r="DX1" s="2">
-        <v>45170</v>
+        <v>45181</v>
       </c>
       <c r="DY1" s="2">
-        <v>45200</v>
+        <v>45211</v>
       </c>
       <c r="DZ1" s="2">
-        <v>45231</v>
+        <v>45240</v>
       </c>
       <c r="EA1" s="2">
-        <v>45261</v>
+        <v>45273</v>
       </c>
       <c r="EB1" s="2">
-        <v>45292</v>
+        <v>45309</v>
       </c>
       <c r="EC1" s="2">
-        <v>45323</v>
+        <v>45331</v>
       </c>
       <c r="ED1" s="2">
-        <v>45352</v>
+        <v>45363</v>
       </c>
       <c r="EE1" s="2">
-        <v>45383</v>
+        <v>45393</v>
       </c>
       <c r="EF1" s="2">
-        <v>45413</v>
+        <v>45422</v>
       </c>
       <c r="EG1" s="2">
-        <v>45444</v>
+        <v>45454</v>
       </c>
       <c r="EH1" s="2">
-        <v>45474</v>
+        <v>45484</v>
       </c>
       <c r="EI1" s="2">
-        <v>45505</v>
+        <v>45517</v>
       </c>
       <c r="EJ1" s="2">
-        <v>45536</v>
+        <v>45547</v>
       </c>
       <c r="EK1" s="2">
-        <v>45566</v>
+        <v>45575</v>
       </c>
       <c r="EL1" s="2">
-        <v>45597</v>
+        <v>45608</v>
       </c>
       <c r="EM1" s="2">
-        <v>45627</v>
+        <v>45638</v>
       </c>
       <c r="EN1" s="2">
-        <v>45658</v>
+        <v>45680</v>
       </c>
       <c r="EO1" s="2">
-        <v>45689</v>
+        <v>45701</v>
       </c>
       <c r="EP1" s="2">
-        <v>45717</v>
+        <v>45729</v>
       </c>
       <c r="EQ1" s="2">
-        <v>45748</v>
+        <v>45758</v>
       </c>
       <c r="ER1" s="2">
-        <v>45778</v>
+        <v>45791</v>
       </c>
       <c r="ES1" s="2">
-        <v>45809</v>
+        <v>45818</v>
       </c>
       <c r="ET1" s="2">
-        <v>45839</v>
+        <v>45849</v>
       </c>
       <c r="EU1" s="2">
-        <v>45870</v>
+        <v>45883</v>
       </c>
       <c r="EV1" s="2">
-        <v>45901</v>
+        <v>45911</v>
       </c>
       <c r="EW1" s="2">
-        <v>45931</v>
+        <v>45946</v>
       </c>
       <c r="EX1" s="2">
-        <v>45962</v>
+        <v>45975</v>
       </c>
       <c r="EY1" s="2">
-        <v>45992</v>
+        <v>46002</v>
       </c>
       <c r="EZ1" s="2">
-        <v>46023</v>
+        <v>46043</v>
       </c>
       <c r="FA1" s="2">
-        <v>46054</v>
+        <v>46066</v>
       </c>
       <c r="FB1" s="2">
-        <v>46082</v>
+        <v>46093</v>
       </c>
       <c r="FC1" s="2">
-        <v>46113</v>
+        <v>46122</v>
       </c>
       <c r="FD1" s="2">
-        <v>46143</v>
+        <v>46155</v>
       </c>
       <c r="FE1" s="2">
-        <v>46174</v>
+        <v>46183</v>
+      </c>
+      <c r="FF1" s="2">
+        <v>46218</v>
       </c>
     </row>
-    <row r="2" spans="1:161" ht="40" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:162" ht="40" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
@@ -1504,8 +1510,11 @@
       <c r="FE2" s="5">
         <v>14.2333</v>
       </c>
+      <c r="FF2" s="5">
+        <v>15.1036</v>
+      </c>
     </row>
-    <row r="3" spans="1:161" ht="30" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:162" ht="30" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -1986,6 +1995,9 @@
       </c>
       <c r="FE3" s="5">
         <v>12.446199999999999</v>
+      </c>
+      <c r="FF3" s="5">
+        <v>14.704499999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>